<commit_message>
feat(F-NAR-019): polish TREE-DIF-001 et TREE-DIF-014 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-001.xlsx
+++ b/stories/arbres/TREE-DIF-001.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le cri d'une mouette entre dans la cuisine. Le sable mouillé suce le bas de la porte. La maison sent le linge, et le sel. Papa pose les sandales, près du palier. Sarah va arriver, Aniss. Aniss ouvre la paume, vers le rebord. Sa coquille rose y tient, légère. Un point d'écume y reste, blanc. Il ne sèche pas. Tu l'as vue, cette petite tache ? Je veux la montrer à Sarah. Au bord de l'eau. En ce moment, des pas sonnent dehors. Aniss, me voilà. Sarah s'arrête, sans un mot. Viens, on court ! Sarah ne bouge pas. Merci, tu as vu son silence. On prépare le sac, alors ?</t>
+          <t>Le cri d'une mouette entre dans la cuisine. Le sable mouillé suce le bas de la porte. Une ombre d'aile passe sur la table. La maison sent le linge, et le sel. Papa pose les sandales, près du palier. Sarah va arriver, Aniss. Aniss ouvre la paume, vers le rebord. C'est le rebord du volet, face à l'eau. Sa coquille rose y tient, légère. Un point d'écume y reste, blanc. Il ne sèche pas. Tu l'as vue, cette petite tache ? Je veux la montrer à Sarah. Au bord de l'eau. En ce moment, des pas sonnent dehors. Aniss, me voilà. Sarah s'arrête, sans un mot. Viens, on court ! Sarah ne bouge pas. Aniss sent ça, dans sa poitrine. On va au bord, ensemble. Merci, tu as vu son silence. On prépare le sac, alors ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cri d'une mouette entre dans la cuisine. Le sable mouillé suce le bas de la porte. La maison sent le linge, et le sel. Papa pose les sandales, près du palier. Sarah va arriver, Aniss. Aniss ouvre la paume, vers le rebord. Sa coquille rose y tient, légère. Un &lt;emphasis level="moderate"&gt;point d'écume&lt;/emphasis&gt; y reste, blanc. Il ne sèche pas. Tu l'as vue, cette petite tache ? Je veux la montrer à Sarah. Au bord de l'eau. En ce moment, des pas sonnent dehors. Aniss, me voilà. Sarah s'arrête, sans un mot. Viens, on court ! Sarah ne bouge pas. Merci, tu as vu son silence. On prépare le sac, alors ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cri d'une mouette entre dans la cuisine. Le sable mouillé suce le bas de la porte. Une ombre d'aile passe sur la table. La maison sent le linge, et le sel. Papa pose les sandales, près du palier. Sarah va arriver, Aniss. Aniss ouvre la paume, vers le rebord. C'est le rebord du volet, face à l'eau. Sa coquille rose y tient, légère. Un &lt;emphasis level="moderate"&gt;point d'écume&lt;/emphasis&gt; y reste, blanc. Il ne sèche pas. Tu l'as vue, cette petite tache ? Je veux la montrer à Sarah. Au bord de l'eau. En ce moment, des pas sonnent dehors. Aniss, me voilà. Sarah s'arrête, sans un mot. Viens, on court ! Sarah ne bouge pas. Aniss sent ça, dans sa poitrine. On va au bord, ensemble. Merci, tu as vu son silence. On prépare le sac, alors ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le cri d'une mouette entre dans la cuisine. Le sable mouillé suce le bas de la porte. La maison sent le linge, et le sel. Papa pose les sandales, près du palier. Sarah va arriver, Aniss. Aniss ouvre la paume, vers le rebord. Sa coquille rose y tient, légère. Un &lt;emphasis&gt;point d'écume&lt;/emphasis&gt; y reste, blanc. Il ne sèche pas. Tu l'as vue, cette petite tache ? Je veux la montrer à Sarah. Au bord de l'eau. En ce moment, des pas sonnent dehors. Aniss, me voilà. Sarah s'arrête, sans un mot. Viens, on court ! Sarah ne bouge pas. Merci, tu as vu son silence. On prépare le sac, alors ? [pause]</t>
+          <t>Le cri d'une mouette entre dans la cuisine. Le sable mouillé suce le bas de la porte. Une ombre d'aile passe sur la table. La maison sent le linge, et le sel. Papa pose les sandales, près du palier. Sarah va arriver, Aniss. Aniss ouvre la paume, vers le rebord. C'est le rebord du volet, face à l'eau. Sa coquille rose y tient, légère. Un &lt;emphasis&gt;point d'écume&lt;/emphasis&gt; y reste, blanc. Il ne sèche pas. Tu l'as vue, cette petite tache ? Je veux la montrer à Sarah. Au bord de l'eau. En ce moment, des pas sonnent dehors. Aniss, me voilà. Sarah s'arrête, sans un mot. Viens, on court ! Sarah ne bouge pas. Aniss sent ça, dans sa poitrine. On va au bord, ensemble. Merci, tu as vu son silence. On prépare le sac, alors ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1343,10 +1343,12 @@
         <is>
           <t>narrateur|Le cri d'une mouette entre dans la cuisine.
 narrateur|Le sable mouillé suce le bas de la porte.
+narrateur|Une ombre d'aile passe sur la table.
 narrateur|La maison sent le linge, et le sel.
 narrateur|Papa pose les sandales, près du palier.
 maman|Sarah va arriver, Aniss.
 narrateur|Aniss ouvre la paume, vers le rebord.
+narrateur|C'est le rebord du volet, face à l'eau.
 narrateur|Sa coquille rose y tient, légère.
 narrateur|Un point d'écume y reste, blanc.
 enfant-m|Il ne sèche pas.
@@ -1358,6 +1360,8 @@
 narrateur|Sarah s'arrête, sans un mot.
 enfant-m|Viens, on court !
 narrateur|Sarah ne bouge pas.
+narrateur|Aniss sent ça, dans sa poitrine.
+enfant-m|On va au bord, ensemble.
 papa|Merci, tu as vu son silence.
 maman|On prépare le sac, alors ?</t>
         </is>
@@ -1391,17 +1395,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Le sac attend, près des sandales. Le seau, le filet, et le linge. Tu prends quoi d'abord, Aniss ?</t>
+          <t>Le sac attend, près des sandales. Le seau, le filet, et le linge. Aniss serre la coquille, puis la pose. Tu prends quoi d'abord, Aniss ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le sac attend, près des sandales. Le seau, le filet, et le linge. Tu prends quoi d'abord, Aniss ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le sac attend, près des sandales. Le seau, le filet, et le linge. Aniss serre la coquille, puis la pose. Tu prends quoi d'abord, Aniss ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le sac attend, près des sandales. Le seau, le filet, et le linge. Tu prends quoi d'abord, Aniss ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le sac attend, près des sandales. Le seau, le filet, et le linge. Aniss serre la coquille, puis la pose. Tu prends quoi d'abord, Aniss ?&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1561,6 +1565,7 @@
         <is>
           <t>narrateur|Le sac attend, près des sandales.
 narrateur|Le seau, le filet, et le linge.
+narrateur|Aniss serre la coquille, puis la pose.
 maman|Tu prends quoi d'abord, Aniss ?</t>
         </is>
       </c>
@@ -17516,7 +17521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17629,6 +17634,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): polish TREE-DIF-001 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-001.xlsx
+++ b/stories/arbres/TREE-DIF-001.xlsx
@@ -17521,7 +17521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17641,6 +17641,13 @@
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>